<commit_message>
#5 IC Part no Changed in Client BOM.
</commit_message>
<xml_diff>
--- a/Design Files/BLE_product-v1.0/BOM/BOM_For_BLE_product-v1.0.xlsx
+++ b/Design Files/BLE_product-v1.0/BOM/BOM_For_BLE_product-v1.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\raafat-BLEproduct\Design Files\BLE_product-v1.0\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -375,9 +375,6 @@
     <t>TLV73330PDQNR</t>
   </si>
   <si>
-    <t>FAN54120UC420X</t>
-  </si>
-  <si>
     <t>CSD25501F3</t>
   </si>
   <si>
@@ -496,6 +493,9 @@
   </si>
   <si>
     <t>BLE_product-v1.0</t>
+  </si>
+  <si>
+    <t>FAN54120MP420X</t>
   </si>
 </sst>
 </file>
@@ -1007,6 +1007,12 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1015,12 +1021,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1389,9 +1389,9 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
+      <c r="J1" s="57"/>
+      <c r="K1" s="57"/>
+      <c r="L1" s="57"/>
     </row>
     <row r="2" spans="1:12" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="51" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
@@ -1420,14 +1420,14 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="52" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
-      <c r="L3" s="56"/>
+      <c r="L3" s="58"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1438,14 +1438,14 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="53" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
-      <c r="L4" s="57"/>
+      <c r="L4" s="59"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1463,7 +1463,7 @@
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
-      <c r="L5" s="57"/>
+      <c r="L5" s="59"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1477,7 +1477,7 @@
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
-      <c r="L6" s="57"/>
+      <c r="L6" s="59"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1491,7 +1491,7 @@
       <c r="I7" s="7"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
-      <c r="L7" s="57"/>
+      <c r="L7" s="59"/>
     </row>
     <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1505,7 +1505,7 @@
       <c r="I8" s="7"/>
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
-      <c r="L8" s="57"/>
+      <c r="L8" s="59"/>
     </row>
     <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1528,19 +1528,19 @@
         <v>99</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I9" s="29" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J9" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="K9" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="L9" s="29" t="s">
         <v>152</v>
-      </c>
-      <c r="K9" s="29" t="s">
-        <v>151</v>
-      </c>
-      <c r="L9" s="29" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1549,7 +1549,7 @@
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="58" t="s">
+      <c r="C10" s="55" t="s">
         <v>7</v>
       </c>
       <c r="D10" s="36" t="s">
@@ -1565,13 +1565,13 @@
         <v>100</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I10" s="36" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J10" s="37" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K10" s="36">
         <v>6</v>
@@ -1584,7 +1584,7 @@
         <f t="shared" ref="B11:B37" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="58" t="s">
+      <c r="C11" s="55" t="s">
         <v>7</v>
       </c>
       <c r="D11" s="38" t="s">
@@ -1600,13 +1600,13 @@
         <v>101</v>
       </c>
       <c r="H11" s="38" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I11" s="38" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J11" s="39" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K11" s="38">
         <v>1</v>
@@ -1619,7 +1619,7 @@
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="59" t="s">
+      <c r="C12" s="56" t="s">
         <v>7</v>
       </c>
       <c r="D12" s="36" t="s">
@@ -1635,13 +1635,13 @@
         <v>102</v>
       </c>
       <c r="H12" s="36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J12" s="37" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K12" s="36">
         <v>1</v>
@@ -1654,7 +1654,7 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="58" t="s">
+      <c r="C13" s="55" t="s">
         <v>7</v>
       </c>
       <c r="D13" s="38" t="s">
@@ -1670,13 +1670,13 @@
         <v>103</v>
       </c>
       <c r="H13" s="38" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I13" s="38" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J13" s="39" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K13" s="38">
         <v>1</v>
@@ -1689,7 +1689,7 @@
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="59" t="s">
+      <c r="C14" s="56" t="s">
         <v>7</v>
       </c>
       <c r="D14" s="36" t="s">
@@ -1705,13 +1705,13 @@
         <v>104</v>
       </c>
       <c r="H14" s="36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I14" s="36" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J14" s="37" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K14" s="36">
         <v>1</v>
@@ -1724,7 +1724,7 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="58" t="s">
+      <c r="C15" s="55" t="s">
         <v>7</v>
       </c>
       <c r="D15" s="38" t="s">
@@ -1740,13 +1740,13 @@
         <v>80</v>
       </c>
       <c r="H15" s="38" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I15" s="38" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J15" s="39" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="K15" s="38">
         <v>1</v>
@@ -1759,7 +1759,7 @@
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
-      <c r="C16" s="59" t="s">
+      <c r="C16" s="56" t="s">
         <v>7</v>
       </c>
       <c r="D16" s="36" t="s">
@@ -1775,13 +1775,13 @@
         <v>105</v>
       </c>
       <c r="H16" s="36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I16" s="36" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J16" s="37" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K16" s="36">
         <v>1</v>
@@ -1794,7 +1794,7 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="58" t="s">
+      <c r="C17" s="55" t="s">
         <v>8</v>
       </c>
       <c r="D17" s="38" t="s">
@@ -1810,11 +1810,11 @@
         <v>81</v>
       </c>
       <c r="H17" s="38" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I17" s="38"/>
       <c r="J17" s="39" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K17" s="38">
         <v>4</v>
@@ -1827,7 +1827,7 @@
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
-      <c r="C18" s="59" t="s">
+      <c r="C18" s="56" t="s">
         <v>9</v>
       </c>
       <c r="D18" s="36" t="s">
@@ -1843,13 +1843,13 @@
         <v>82</v>
       </c>
       <c r="H18" s="36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I18" s="36" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J18" s="37" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K18" s="36">
         <v>1</v>
@@ -1862,7 +1862,7 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="58" t="s">
+      <c r="C19" s="55" t="s">
         <v>10</v>
       </c>
       <c r="D19" s="38" t="s">
@@ -1878,11 +1878,11 @@
         <v>106</v>
       </c>
       <c r="H19" s="38" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I19" s="38"/>
       <c r="J19" s="39" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K19" s="38">
         <v>1</v>
@@ -1895,8 +1895,8 @@
         <f>ROW(B20) - ROW($B$9)</f>
         <v>11</v>
       </c>
-      <c r="C20" s="59" t="s">
-        <v>156</v>
+      <c r="C20" s="56" t="s">
+        <v>155</v>
       </c>
       <c r="D20" s="36" t="s">
         <v>28</v>
@@ -1907,11 +1907,11 @@
       </c>
       <c r="G20" s="37"/>
       <c r="H20" s="36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I20" s="36"/>
       <c r="J20" s="37" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K20" s="36">
         <v>1</v>
@@ -1924,7 +1924,7 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="58" t="s">
+      <c r="C21" s="55" t="s">
         <v>11</v>
       </c>
       <c r="D21" s="38" t="s">
@@ -1940,13 +1940,13 @@
         <v>107</v>
       </c>
       <c r="H21" s="38" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I21" s="38" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J21" s="39" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K21" s="38">
         <v>1</v>
@@ -1959,7 +1959,7 @@
         <f>ROW(B22) - ROW($B$9)</f>
         <v>13</v>
       </c>
-      <c r="C22" s="59" t="s">
+      <c r="C22" s="56" t="s">
         <v>12</v>
       </c>
       <c r="D22" s="36" t="s">
@@ -1975,13 +1975,13 @@
         <v>86</v>
       </c>
       <c r="H22" s="36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I22" s="36" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="J22" s="37" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K22" s="36">
         <v>1</v>
@@ -1994,7 +1994,7 @@
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="58" t="s">
+      <c r="C23" s="55" t="s">
         <v>13</v>
       </c>
       <c r="D23" s="38" t="s">
@@ -2010,13 +2010,13 @@
         <v>108</v>
       </c>
       <c r="H23" s="38" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I23" s="38" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J23" s="39" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K23" s="38">
         <v>1</v>
@@ -2029,7 +2029,7 @@
         <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
       </c>
-      <c r="C24" s="59" t="s">
+      <c r="C24" s="56" t="s">
         <v>14</v>
       </c>
       <c r="D24" s="36" t="s">
@@ -2045,13 +2045,13 @@
         <v>109</v>
       </c>
       <c r="H24" s="36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I24" s="36" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J24" s="37" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K24" s="36">
         <v>5</v>
@@ -2064,7 +2064,7 @@
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="58" t="s">
+      <c r="C25" s="55" t="s">
         <v>14</v>
       </c>
       <c r="D25" s="38" t="s">
@@ -2080,13 +2080,13 @@
         <v>110</v>
       </c>
       <c r="H25" s="38" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I25" s="38" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J25" s="39" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="K25" s="38">
         <v>1</v>
@@ -2099,7 +2099,7 @@
         <f>ROW(B26) - ROW($B$9)</f>
         <v>17</v>
       </c>
-      <c r="C26" s="59" t="s">
+      <c r="C26" s="56" t="s">
         <v>14</v>
       </c>
       <c r="D26" s="36" t="s">
@@ -2115,13 +2115,13 @@
         <v>111</v>
       </c>
       <c r="H26" s="36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I26" s="36" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J26" s="37" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="K26" s="36">
         <v>1</v>
@@ -2134,7 +2134,7 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C27" s="58" t="s">
+      <c r="C27" s="55" t="s">
         <v>14</v>
       </c>
       <c r="D27" s="38" t="s">
@@ -2150,13 +2150,13 @@
         <v>112</v>
       </c>
       <c r="H27" s="38" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I27" s="38" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J27" s="39" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="K27" s="38">
         <v>2</v>
@@ -2169,7 +2169,7 @@
         <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
-      <c r="C28" s="59" t="s">
+      <c r="C28" s="56" t="s">
         <v>14</v>
       </c>
       <c r="D28" s="36" t="s">
@@ -2185,13 +2185,13 @@
         <v>113</v>
       </c>
       <c r="H28" s="36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I28" s="36" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J28" s="37" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="K28" s="36">
         <v>4</v>
@@ -2204,7 +2204,7 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C29" s="58" t="s">
+      <c r="C29" s="55" t="s">
         <v>15</v>
       </c>
       <c r="D29" s="38" t="s">
@@ -2220,13 +2220,13 @@
         <v>114</v>
       </c>
       <c r="H29" s="38" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I29" s="38" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="J29" s="39" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K29" s="38">
         <v>1</v>
@@ -2239,7 +2239,7 @@
         <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
       </c>
-      <c r="C30" s="59" t="s">
+      <c r="C30" s="56" t="s">
         <v>16</v>
       </c>
       <c r="D30" s="36" t="s">
@@ -2255,13 +2255,13 @@
         <v>115</v>
       </c>
       <c r="H30" s="36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I30" s="36" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J30" s="37" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K30" s="36">
         <v>1</v>
@@ -2274,7 +2274,7 @@
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C31" s="58" t="s">
+      <c r="C31" s="55" t="s">
         <v>16</v>
       </c>
       <c r="D31" s="38" t="s">
@@ -2290,13 +2290,13 @@
         <v>116</v>
       </c>
       <c r="H31" s="38" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I31" s="38" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J31" s="39" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K31" s="38">
         <v>1</v>
@@ -2309,7 +2309,7 @@
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="59" t="s">
+      <c r="C32" s="56" t="s">
         <v>16</v>
       </c>
       <c r="D32" s="36" t="s">
@@ -2325,13 +2325,13 @@
         <v>117</v>
       </c>
       <c r="H32" s="36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I32" s="36" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="J32" s="37" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K32" s="36">
         <v>1</v>
@@ -2344,7 +2344,7 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C33" s="58" t="s">
+      <c r="C33" s="55" t="s">
         <v>16</v>
       </c>
       <c r="D33" s="38" t="s">
@@ -2357,16 +2357,16 @@
         <v>93</v>
       </c>
       <c r="G33" s="39" t="s">
-        <v>118</v>
+        <v>158</v>
       </c>
       <c r="H33" s="38" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I33" s="38" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J33" s="39" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K33" s="38">
         <v>1</v>
@@ -2379,7 +2379,7 @@
         <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
-      <c r="C34" s="59" t="s">
+      <c r="C34" s="56" t="s">
         <v>16</v>
       </c>
       <c r="D34" s="36" t="s">
@@ -2392,16 +2392,16 @@
         <v>94</v>
       </c>
       <c r="G34" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H34" s="36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I34" s="36" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="J34" s="37" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K34" s="36">
         <v>1</v>
@@ -2414,7 +2414,7 @@
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C35" s="58" t="s">
+      <c r="C35" s="55" t="s">
         <v>16</v>
       </c>
       <c r="D35" s="38" t="s">
@@ -2430,13 +2430,13 @@
         <v>95</v>
       </c>
       <c r="H35" s="38" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I35" s="38" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J35" s="39" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K35" s="38">
         <v>1</v>
@@ -2449,7 +2449,7 @@
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
-      <c r="C36" s="59" t="s">
+      <c r="C36" s="56" t="s">
         <v>16</v>
       </c>
       <c r="D36" s="36" t="s">
@@ -2462,16 +2462,16 @@
         <v>96</v>
       </c>
       <c r="G36" s="37" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H36" s="36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I36" s="36" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="J36" s="37" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K36" s="36">
         <v>1</v>
@@ -2484,7 +2484,7 @@
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C37" s="58" t="s">
+      <c r="C37" s="55" t="s">
         <v>16</v>
       </c>
       <c r="D37" s="38" t="s">
@@ -2497,16 +2497,16 @@
         <v>97</v>
       </c>
       <c r="G37" s="39" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H37" s="38" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I37" s="38" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="J37" s="39" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K37" s="38">
         <v>1</v>
@@ -2519,7 +2519,7 @@
         <f>ROW(B38) - ROW($B$9)</f>
         <v>29</v>
       </c>
-      <c r="C38" s="59" t="s">
+      <c r="C38" s="56" t="s">
         <v>16</v>
       </c>
       <c r="D38" s="36" t="s">
@@ -2532,16 +2532,16 @@
         <v>98</v>
       </c>
       <c r="G38" s="37" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H38" s="36" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="I38" s="36" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="J38" s="37" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K38" s="36">
         <v>1</v>

</xml_diff>

<commit_message>
#5 Client BOM updated.
</commit_message>
<xml_diff>
--- a/Design Files/BLE_product-v1.0/BOM/BOM_For_BLE_product-v1.0.xlsx
+++ b/Design Files/BLE_product-v1.0/BOM/BOM_For_BLE_product-v1.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="168">
   <si>
     <t>Component list</t>
   </si>
@@ -273,9 +273,6 @@
     <t>Sensor-Pads 0.5mm Dia</t>
   </si>
   <si>
-    <t>TC2030-IDC-NL_</t>
-  </si>
-  <si>
     <t>IND-0806</t>
   </si>
   <si>
@@ -496,6 +493,37 @@
   </si>
   <si>
     <t>FAN54120MP420X</t>
+  </si>
+  <si>
+    <t>Peripherals</t>
+  </si>
+  <si>
+    <t>dc2.0*0.5mm USB Charger Cable Small Pin Charging Cord</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>Do Not Mount</t>
+  </si>
+  <si>
+    <t>Aliexpress</t>
+  </si>
+  <si>
+    <t>TC2030-IDC-NL</t>
+  </si>
+  <si>
+    <t>“No Legs” 6-pin Plug-of-Nails™ Cable fitted with a 6-pin 0.1″ pitch ribbon connector.</t>
+  </si>
+  <si>
+    <t>Tag Connect</t>
+  </si>
+  <si>
+    <t>USB DC 2.0*0.5mm Charging Cable for Mini S530 Smallest Invisible Wireless Bluetooth Earbuds Earphones Headphones Headset</t>
+  </si>
+  <si>
+    <t xml:space="preserve">“No Legs” 6-pin Plug-of-Nails™ Cable fitted with a 6-pin 0.1″ pitch ribbon connector.
+</t>
   </si>
 </sst>
 </file>
@@ -505,7 +533,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -636,6 +664,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -663,7 +707,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -858,11 +902,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1022,8 +1093,40 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1049,13 +1152,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>11</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>47625</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>19942</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
+      <xdr:col>12</xdr:col>
       <xdr:colOff>1905000</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>171450</xdr:rowOff>
@@ -1363,7 +1466,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:M43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -1375,11 +1478,12 @@
     <col min="8" max="8" width="22" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="29.42578125" customWidth="1"/>
+    <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1392,8 +1496,9 @@
       <c r="J1" s="57"/>
       <c r="K1" s="57"/>
       <c r="L1" s="57"/>
-    </row>
-    <row r="2" spans="1:12" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M1" s="57"/>
+    </row>
+    <row r="2" spans="1:13" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="20"/>
       <c r="C2" s="43"/>
@@ -1402,16 +1507,17 @@
       </c>
       <c r="E2" s="10"/>
       <c r="F2" s="51" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G2" s="11"/>
       <c r="H2" s="11"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
       <c r="K2" s="3"/>
-      <c r="L2" s="40"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L2" s="3"/>
+      <c r="M2" s="40"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="21"/>
       <c r="C3" s="44"/>
@@ -1420,16 +1526,17 @@
       </c>
       <c r="E3" s="12"/>
       <c r="F3" s="52" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
-      <c r="L3" s="58"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L3" s="4"/>
+      <c r="M3" s="58"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="21"/>
       <c r="C4" s="44"/>
@@ -1438,16 +1545,17 @@
       </c>
       <c r="E4" s="12"/>
       <c r="F4" s="53" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G4" s="13"/>
       <c r="H4" s="13"/>
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
-      <c r="L4" s="59"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L4" s="6"/>
+      <c r="M4" s="59"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="21"/>
       <c r="C5" s="44"/>
@@ -1463,9 +1571,10 @@
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
-      <c r="L5" s="59"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L5" s="5"/>
+      <c r="M5" s="59"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="22"/>
       <c r="C6" s="45"/>
@@ -1477,9 +1586,10 @@
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
-      <c r="L6" s="59"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L6" s="5"/>
+      <c r="M6" s="59"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="23"/>
       <c r="C7" s="46"/>
@@ -1491,9 +1601,10 @@
       <c r="I7" s="7"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
-      <c r="L7" s="59"/>
-    </row>
-    <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L7" s="7"/>
+      <c r="M7" s="59"/>
+    </row>
+    <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="26"/>
       <c r="C8" s="47"/>
@@ -1505,9 +1616,10 @@
       <c r="I8" s="7"/>
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
-      <c r="L8" s="59"/>
-    </row>
-    <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="L8" s="7"/>
+      <c r="M8" s="59"/>
+    </row>
+    <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="29" t="s">
         <v>4</v>
@@ -1525,25 +1637,28 @@
         <v>76</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="I9" s="29" t="s">
-        <v>122</v>
-      </c>
-      <c r="J9" s="30" t="s">
+        <v>121</v>
+      </c>
+      <c r="J9" s="29" t="s">
+        <v>150</v>
+      </c>
+      <c r="K9" s="30" t="s">
+        <v>160</v>
+      </c>
+      <c r="L9" s="29" t="s">
+        <v>149</v>
+      </c>
+      <c r="M9" s="29" t="s">
         <v>151</v>
       </c>
-      <c r="K9" s="29" t="s">
-        <v>150</v>
-      </c>
-      <c r="L9" s="29" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="50">
         <f>ROW(B10) - ROW($B$9)</f>
@@ -1562,23 +1677,24 @@
         <v>77</v>
       </c>
       <c r="G10" s="37" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H10" s="36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I10" s="36" t="s">
-        <v>123</v>
-      </c>
-      <c r="J10" s="37" t="s">
-        <v>138</v>
-      </c>
-      <c r="K10" s="36">
+        <v>122</v>
+      </c>
+      <c r="J10" s="36" t="s">
+        <v>137</v>
+      </c>
+      <c r="K10" s="61"/>
+      <c r="L10" s="36">
         <v>6</v>
       </c>
-      <c r="L10" s="36"/>
-    </row>
-    <row r="11" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M10" s="36"/>
+    </row>
+    <row r="11" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="50">
         <f t="shared" ref="B11:B37" si="0">ROW(B11) - ROW($B$9)</f>
@@ -1597,23 +1713,24 @@
         <v>78</v>
       </c>
       <c r="G11" s="39" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H11" s="38" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I11" s="38" t="s">
-        <v>124</v>
-      </c>
-      <c r="J11" s="39" t="s">
-        <v>139</v>
-      </c>
-      <c r="K11" s="38">
+        <v>123</v>
+      </c>
+      <c r="J11" s="38" t="s">
+        <v>138</v>
+      </c>
+      <c r="K11" s="62"/>
+      <c r="L11" s="38">
         <v>1</v>
       </c>
-      <c r="L11" s="38"/>
-    </row>
-    <row r="12" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M11" s="38"/>
+    </row>
+    <row r="12" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="50">
         <f>ROW(B12) - ROW($B$9)</f>
@@ -1632,23 +1749,24 @@
         <v>79</v>
       </c>
       <c r="G12" s="37" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H12" s="36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I12" s="36" t="s">
-        <v>123</v>
-      </c>
-      <c r="J12" s="37" t="s">
-        <v>140</v>
-      </c>
-      <c r="K12" s="36">
+        <v>122</v>
+      </c>
+      <c r="J12" s="36" t="s">
+        <v>139</v>
+      </c>
+      <c r="K12" s="61"/>
+      <c r="L12" s="36">
         <v>1</v>
       </c>
-      <c r="L12" s="36"/>
-    </row>
-    <row r="13" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M12" s="36"/>
+    </row>
+    <row r="13" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="50">
         <f t="shared" si="0"/>
@@ -1667,23 +1785,24 @@
         <v>77</v>
       </c>
       <c r="G13" s="39" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H13" s="38" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I13" s="38" t="s">
-        <v>123</v>
-      </c>
-      <c r="J13" s="39" t="s">
-        <v>141</v>
-      </c>
-      <c r="K13" s="38">
+        <v>122</v>
+      </c>
+      <c r="J13" s="38" t="s">
+        <v>140</v>
+      </c>
+      <c r="K13" s="62"/>
+      <c r="L13" s="38">
         <v>1</v>
       </c>
-      <c r="L13" s="38"/>
-    </row>
-    <row r="14" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M13" s="38"/>
+    </row>
+    <row r="14" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="50">
         <f>ROW(B14) - ROW($B$9)</f>
@@ -1702,23 +1821,24 @@
         <v>77</v>
       </c>
       <c r="G14" s="37" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H14" s="36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I14" s="36" t="s">
-        <v>123</v>
-      </c>
-      <c r="J14" s="37" t="s">
-        <v>142</v>
-      </c>
-      <c r="K14" s="36">
+        <v>122</v>
+      </c>
+      <c r="J14" s="36" t="s">
+        <v>141</v>
+      </c>
+      <c r="K14" s="63"/>
+      <c r="L14" s="36">
         <v>1</v>
       </c>
-      <c r="L14" s="36"/>
-    </row>
-    <row r="15" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M14" s="36"/>
+    </row>
+    <row r="15" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="50">
         <f t="shared" si="0"/>
@@ -1740,20 +1860,21 @@
         <v>80</v>
       </c>
       <c r="H15" s="38" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I15" s="38" t="s">
-        <v>125</v>
-      </c>
-      <c r="J15" s="39" t="s">
-        <v>143</v>
-      </c>
-      <c r="K15" s="38">
+        <v>124</v>
+      </c>
+      <c r="J15" s="38" t="s">
+        <v>142</v>
+      </c>
+      <c r="K15" s="62"/>
+      <c r="L15" s="38">
         <v>1</v>
       </c>
-      <c r="L15" s="38"/>
-    </row>
-    <row r="16" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M15" s="38"/>
+    </row>
+    <row r="16" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="50">
         <f>ROW(B16) - ROW($B$9)</f>
@@ -1772,23 +1893,24 @@
         <v>77</v>
       </c>
       <c r="G16" s="37" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H16" s="36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I16" s="36" t="s">
-        <v>123</v>
-      </c>
-      <c r="J16" s="37" t="s">
-        <v>141</v>
-      </c>
-      <c r="K16" s="36">
+        <v>122</v>
+      </c>
+      <c r="J16" s="36" t="s">
+        <v>140</v>
+      </c>
+      <c r="K16" s="63"/>
+      <c r="L16" s="36">
         <v>1</v>
       </c>
-      <c r="L16" s="36"/>
-    </row>
-    <row r="17" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M16" s="36"/>
+    </row>
+    <row r="17" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="50">
         <f t="shared" si="0"/>
@@ -1810,18 +1932,23 @@
         <v>81</v>
       </c>
       <c r="H17" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="I17" s="38"/>
-      <c r="J17" s="39" t="s">
-        <v>154</v>
-      </c>
-      <c r="K17" s="38">
+        <v>153</v>
+      </c>
+      <c r="I17" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="J17" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="K17" s="36"/>
+      <c r="L17" s="38">
         <v>4</v>
       </c>
-      <c r="L17" s="38"/>
-    </row>
-    <row r="18" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M17" s="64" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="50">
         <f>ROW(B18) - ROW($B$9)</f>
@@ -1843,20 +1970,21 @@
         <v>82</v>
       </c>
       <c r="H18" s="36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I18" s="36" t="s">
-        <v>126</v>
-      </c>
-      <c r="J18" s="37" t="s">
-        <v>154</v>
-      </c>
-      <c r="K18" s="36">
+        <v>125</v>
+      </c>
+      <c r="J18" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="K18" s="61"/>
+      <c r="L18" s="36">
         <v>1</v>
       </c>
-      <c r="L18" s="36"/>
-    </row>
-    <row r="19" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M18" s="36"/>
+    </row>
+    <row r="19" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="50">
         <f t="shared" si="0"/>
@@ -1875,50 +2003,64 @@
         <v>83</v>
       </c>
       <c r="G19" s="39" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H19" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="I19" s="38"/>
-      <c r="J19" s="39" t="s">
-        <v>154</v>
-      </c>
-      <c r="K19" s="38">
+        <v>153</v>
+      </c>
+      <c r="I19" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="J19" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="K19" s="36"/>
+      <c r="L19" s="38">
         <v>1</v>
       </c>
-      <c r="L19" s="38"/>
-    </row>
-    <row r="20" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M19" s="64" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="50">
         <f>ROW(B20) - ROW($B$9)</f>
         <v>11</v>
       </c>
       <c r="C20" s="56" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D20" s="36" t="s">
         <v>28</v>
       </c>
-      <c r="E20" s="37"/>
+      <c r="E20" s="37" t="s">
+        <v>164</v>
+      </c>
       <c r="F20" s="36" t="s">
-        <v>84</v>
-      </c>
-      <c r="G20" s="37"/>
+        <v>153</v>
+      </c>
+      <c r="G20" s="36" t="s">
+        <v>163</v>
+      </c>
       <c r="H20" s="36" t="s">
-        <v>154</v>
-      </c>
-      <c r="I20" s="36"/>
-      <c r="J20" s="37" t="s">
-        <v>154</v>
-      </c>
-      <c r="K20" s="36">
+        <v>153</v>
+      </c>
+      <c r="I20" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="J20" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="K20" s="61"/>
+      <c r="L20" s="36">
         <v>1</v>
       </c>
-      <c r="L20" s="36"/>
-    </row>
-    <row r="21" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M20" s="64" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="50">
         <f t="shared" si="0"/>
@@ -1934,26 +2076,27 @@
         <v>58</v>
       </c>
       <c r="F21" s="38" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G21" s="39" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H21" s="38" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I21" s="38" t="s">
-        <v>127</v>
-      </c>
-      <c r="J21" s="39" t="s">
-        <v>144</v>
-      </c>
-      <c r="K21" s="38">
+        <v>126</v>
+      </c>
+      <c r="J21" s="38" t="s">
+        <v>143</v>
+      </c>
+      <c r="K21" s="61"/>
+      <c r="L21" s="38">
         <v>1</v>
       </c>
-      <c r="L21" s="38"/>
-    </row>
-    <row r="22" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M21" s="38"/>
+    </row>
+    <row r="22" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="50">
         <f>ROW(B22) - ROW($B$9)</f>
@@ -1969,26 +2112,27 @@
         <v>59</v>
       </c>
       <c r="F22" s="36" t="s">
-        <v>86</v>
+        <v>153</v>
       </c>
       <c r="G22" s="37" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H22" s="36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I22" s="36" t="s">
-        <v>128</v>
-      </c>
-      <c r="J22" s="37" t="s">
-        <v>154</v>
-      </c>
-      <c r="K22" s="36">
+        <v>127</v>
+      </c>
+      <c r="J22" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="K22" s="36"/>
+      <c r="L22" s="36">
         <v>1</v>
       </c>
-      <c r="L22" s="36"/>
-    </row>
-    <row r="23" spans="1:12" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M22" s="36"/>
+    </row>
+    <row r="23" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="50">
         <f t="shared" si="0"/>
@@ -2004,26 +2148,27 @@
         <v>60</v>
       </c>
       <c r="F23" s="38" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G23" s="39" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H23" s="38" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I23" s="38" t="s">
-        <v>129</v>
-      </c>
-      <c r="J23" s="39" t="s">
-        <v>154</v>
-      </c>
-      <c r="K23" s="38">
+        <v>128</v>
+      </c>
+      <c r="J23" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="K23" s="38"/>
+      <c r="L23" s="38">
         <v>1</v>
       </c>
-      <c r="L23" s="38"/>
-    </row>
-    <row r="24" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M23" s="38"/>
+    </row>
+    <row r="24" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="50">
         <f>ROW(B24) - ROW($B$9)</f>
@@ -2039,26 +2184,27 @@
         <v>61</v>
       </c>
       <c r="F24" s="36" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G24" s="37" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H24" s="36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I24" s="36" t="s">
-        <v>123</v>
-      </c>
-      <c r="J24" s="37" t="s">
-        <v>145</v>
-      </c>
-      <c r="K24" s="36">
+        <v>122</v>
+      </c>
+      <c r="J24" s="36" t="s">
+        <v>144</v>
+      </c>
+      <c r="K24" s="62"/>
+      <c r="L24" s="36">
         <v>5</v>
       </c>
-      <c r="L24" s="36"/>
-    </row>
-    <row r="25" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M24" s="36"/>
+    </row>
+    <row r="25" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="50">
         <f t="shared" si="0"/>
@@ -2074,26 +2220,27 @@
         <v>62</v>
       </c>
       <c r="F25" s="38" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G25" s="39" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H25" s="38" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I25" s="38" t="s">
-        <v>130</v>
-      </c>
-      <c r="J25" s="39" t="s">
-        <v>146</v>
-      </c>
-      <c r="K25" s="38">
+        <v>129</v>
+      </c>
+      <c r="J25" s="38" t="s">
+        <v>145</v>
+      </c>
+      <c r="K25" s="38"/>
+      <c r="L25" s="38">
         <v>1</v>
       </c>
-      <c r="L25" s="38"/>
-    </row>
-    <row r="26" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M25" s="38"/>
+    </row>
+    <row r="26" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="50">
         <f>ROW(B26) - ROW($B$9)</f>
@@ -2109,26 +2256,27 @@
         <v>63</v>
       </c>
       <c r="F26" s="36" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G26" s="37" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H26" s="36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I26" s="36" t="s">
-        <v>130</v>
-      </c>
-      <c r="J26" s="37" t="s">
-        <v>147</v>
-      </c>
-      <c r="K26" s="36">
+        <v>129</v>
+      </c>
+      <c r="J26" s="36" t="s">
+        <v>146</v>
+      </c>
+      <c r="K26" s="36"/>
+      <c r="L26" s="36">
         <v>1</v>
       </c>
-      <c r="L26" s="36"/>
-    </row>
-    <row r="27" spans="1:12" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M26" s="36"/>
+    </row>
+    <row r="27" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="50">
         <f t="shared" si="0"/>
@@ -2144,26 +2292,27 @@
         <v>64</v>
       </c>
       <c r="F27" s="38" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G27" s="39" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H27" s="38" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I27" s="38" t="s">
-        <v>130</v>
-      </c>
-      <c r="J27" s="39" t="s">
-        <v>148</v>
-      </c>
-      <c r="K27" s="38">
+        <v>129</v>
+      </c>
+      <c r="J27" s="38" t="s">
+        <v>147</v>
+      </c>
+      <c r="K27" s="38"/>
+      <c r="L27" s="38">
         <v>2</v>
       </c>
-      <c r="L27" s="38"/>
-    </row>
-    <row r="28" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M27" s="38"/>
+    </row>
+    <row r="28" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="50">
         <f>ROW(B28) - ROW($B$9)</f>
@@ -2179,26 +2328,27 @@
         <v>65</v>
       </c>
       <c r="F28" s="36" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G28" s="37" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H28" s="36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I28" s="36" t="s">
-        <v>123</v>
-      </c>
-      <c r="J28" s="37" t="s">
-        <v>149</v>
-      </c>
-      <c r="K28" s="36">
+        <v>122</v>
+      </c>
+      <c r="J28" s="36" t="s">
+        <v>148</v>
+      </c>
+      <c r="K28" s="62"/>
+      <c r="L28" s="36">
         <v>4</v>
       </c>
-      <c r="L28" s="36"/>
-    </row>
-    <row r="29" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M28" s="36"/>
+    </row>
+    <row r="29" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="50">
         <f t="shared" si="0"/>
@@ -2214,26 +2364,27 @@
         <v>66</v>
       </c>
       <c r="F29" s="38" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G29" s="39" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H29" s="38" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I29" s="38" t="s">
-        <v>131</v>
-      </c>
-      <c r="J29" s="39" t="s">
-        <v>154</v>
-      </c>
-      <c r="K29" s="38">
+        <v>130</v>
+      </c>
+      <c r="J29" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="K29" s="61"/>
+      <c r="L29" s="38">
         <v>1</v>
       </c>
-      <c r="L29" s="38"/>
-    </row>
-    <row r="30" spans="1:12" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M29" s="38"/>
+    </row>
+    <row r="30" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="50">
         <f>ROW(B30) - ROW($B$9)</f>
@@ -2249,26 +2400,27 @@
         <v>67</v>
       </c>
       <c r="F30" s="36" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G30" s="37" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H30" s="36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I30" s="36" t="s">
-        <v>132</v>
-      </c>
-      <c r="J30" s="37" t="s">
-        <v>154</v>
-      </c>
-      <c r="K30" s="36">
+        <v>131</v>
+      </c>
+      <c r="J30" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="K30" s="62"/>
+      <c r="L30" s="36">
         <v>1</v>
       </c>
-      <c r="L30" s="36"/>
-    </row>
-    <row r="31" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M30" s="36"/>
+    </row>
+    <row r="31" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="50">
         <f t="shared" si="0"/>
@@ -2284,26 +2436,27 @@
         <v>68</v>
       </c>
       <c r="F31" s="38" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G31" s="39" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H31" s="38" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I31" s="38" t="s">
-        <v>133</v>
-      </c>
-      <c r="J31" s="39" t="s">
-        <v>154</v>
-      </c>
-      <c r="K31" s="38">
+        <v>132</v>
+      </c>
+      <c r="J31" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="K31" s="65"/>
+      <c r="L31" s="38">
         <v>1</v>
       </c>
-      <c r="L31" s="38"/>
-    </row>
-    <row r="32" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M31" s="38"/>
+    </row>
+    <row r="32" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="50">
         <f>ROW(B32) - ROW($B$9)</f>
@@ -2319,26 +2472,27 @@
         <v>69</v>
       </c>
       <c r="F32" s="36" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G32" s="37" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H32" s="36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I32" s="36" t="s">
-        <v>134</v>
-      </c>
-      <c r="J32" s="37" t="s">
-        <v>154</v>
-      </c>
-      <c r="K32" s="36">
+        <v>133</v>
+      </c>
+      <c r="J32" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="K32" s="65"/>
+      <c r="L32" s="36">
         <v>1</v>
       </c>
-      <c r="L32" s="36"/>
-    </row>
-    <row r="33" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M32" s="36"/>
+    </row>
+    <row r="33" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="50">
         <f t="shared" si="0"/>
@@ -2354,26 +2508,27 @@
         <v>70</v>
       </c>
       <c r="F33" s="38" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G33" s="39" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H33" s="38" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I33" s="38" t="s">
-        <v>135</v>
-      </c>
-      <c r="J33" s="39" t="s">
-        <v>154</v>
-      </c>
-      <c r="K33" s="38">
+        <v>134</v>
+      </c>
+      <c r="J33" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="K33" s="65"/>
+      <c r="L33" s="38">
         <v>1</v>
       </c>
-      <c r="L33" s="38"/>
-    </row>
-    <row r="34" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M33" s="38"/>
+    </row>
+    <row r="34" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="50">
         <f>ROW(B34) - ROW($B$9)</f>
@@ -2389,26 +2544,27 @@
         <v>71</v>
       </c>
       <c r="F34" s="36" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G34" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H34" s="36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I34" s="36" t="s">
-        <v>134</v>
-      </c>
-      <c r="J34" s="37" t="s">
-        <v>154</v>
-      </c>
-      <c r="K34" s="36">
+        <v>133</v>
+      </c>
+      <c r="J34" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="K34" s="65"/>
+      <c r="L34" s="36">
         <v>1</v>
       </c>
-      <c r="L34" s="36"/>
-    </row>
-    <row r="35" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M34" s="36"/>
+    </row>
+    <row r="35" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="50">
         <f t="shared" si="0"/>
@@ -2424,26 +2580,27 @@
         <v>72</v>
       </c>
       <c r="F35" s="38" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G35" s="39" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H35" s="38" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I35" s="38" t="s">
-        <v>136</v>
-      </c>
-      <c r="J35" s="39" t="s">
-        <v>154</v>
-      </c>
-      <c r="K35" s="38">
+        <v>135</v>
+      </c>
+      <c r="J35" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="K35" s="65"/>
+      <c r="L35" s="38">
         <v>1</v>
       </c>
-      <c r="L35" s="38"/>
-    </row>
-    <row r="36" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M35" s="38"/>
+    </row>
+    <row r="36" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="50">
         <f>ROW(B36) - ROW($B$9)</f>
@@ -2459,26 +2616,27 @@
         <v>73</v>
       </c>
       <c r="F36" s="36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G36" s="37" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H36" s="36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I36" s="36" t="s">
-        <v>135</v>
-      </c>
-      <c r="J36" s="37" t="s">
-        <v>154</v>
-      </c>
-      <c r="K36" s="36">
+        <v>134</v>
+      </c>
+      <c r="J36" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="K36" s="65"/>
+      <c r="L36" s="36">
         <v>1</v>
       </c>
-      <c r="L36" s="36"/>
-    </row>
-    <row r="37" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M36" s="36"/>
+    </row>
+    <row r="37" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="50">
         <f t="shared" si="0"/>
@@ -2494,26 +2652,27 @@
         <v>74</v>
       </c>
       <c r="F37" s="38" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G37" s="39" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H37" s="38" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I37" s="38" t="s">
-        <v>137</v>
-      </c>
-      <c r="J37" s="39" t="s">
-        <v>154</v>
-      </c>
-      <c r="K37" s="38">
+        <v>136</v>
+      </c>
+      <c r="J37" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="K37" s="65"/>
+      <c r="L37" s="38">
         <v>1</v>
       </c>
-      <c r="L37" s="38"/>
-    </row>
-    <row r="38" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M37" s="38"/>
+    </row>
+    <row r="38" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="50">
         <f>ROW(B38) - ROW($B$9)</f>
@@ -2529,60 +2688,165 @@
         <v>75</v>
       </c>
       <c r="F38" s="36" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G38" s="37" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H38" s="36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I38" s="36" t="s">
-        <v>137</v>
-      </c>
-      <c r="J38" s="37" t="s">
-        <v>154</v>
-      </c>
-      <c r="K38" s="36">
+        <v>136</v>
+      </c>
+      <c r="J38" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="K38" s="65"/>
+      <c r="L38" s="36">
         <v>1</v>
       </c>
-      <c r="L38" s="36"/>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M38" s="36"/>
+    </row>
+    <row r="39" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
-      <c r="B39" s="31"/>
-      <c r="C39" s="48"/>
-      <c r="D39" s="32"/>
-      <c r="E39" s="33"/>
-      <c r="F39" s="34"/>
-      <c r="G39" s="35"/>
-      <c r="H39" s="35"/>
-      <c r="I39" s="34"/>
-      <c r="J39" s="35"/>
-      <c r="K39" s="35"/>
-      <c r="L39" s="41"/>
-    </row>
-    <row r="40" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B39" s="60">
+        <v>30</v>
+      </c>
+      <c r="C39" s="56" t="s">
+        <v>158</v>
+      </c>
+      <c r="D39" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="E39" s="37" t="s">
+        <v>159</v>
+      </c>
+      <c r="F39" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="G39" s="37" t="s">
+        <v>153</v>
+      </c>
+      <c r="H39" s="36"/>
+      <c r="I39" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="J39" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="K39" s="66" t="s">
+        <v>162</v>
+      </c>
+      <c r="L39" s="36">
+        <v>1</v>
+      </c>
+      <c r="M39" s="36"/>
+    </row>
+    <row r="40" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
-      <c r="B40" s="24"/>
-      <c r="C40" s="49"/>
-      <c r="D40" s="8"/>
-      <c r="E40" s="9"/>
-      <c r="F40" s="9"/>
-      <c r="G40" s="9"/>
-      <c r="H40" s="9"/>
-      <c r="I40" s="9"/>
-      <c r="J40" s="9"/>
-      <c r="K40" s="9"/>
-      <c r="L40" s="42"/>
+      <c r="B40" s="60">
+        <v>31</v>
+      </c>
+      <c r="C40" s="56" t="s">
+        <v>158</v>
+      </c>
+      <c r="D40" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="E40" s="37" t="s">
+        <v>166</v>
+      </c>
+      <c r="F40" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="G40" s="37" t="s">
+        <v>153</v>
+      </c>
+      <c r="H40" s="36"/>
+      <c r="I40" s="36" t="s">
+        <v>153</v>
+      </c>
+      <c r="J40" s="67" t="s">
+        <v>153</v>
+      </c>
+      <c r="K40" s="70" t="s">
+        <v>162</v>
+      </c>
+      <c r="L40" s="68">
+        <v>1</v>
+      </c>
+      <c r="M40" s="36"/>
+    </row>
+    <row r="41" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="1"/>
+      <c r="B41" s="60">
+        <v>32</v>
+      </c>
+      <c r="C41" s="56" t="s">
+        <v>158</v>
+      </c>
+      <c r="D41" s="36"/>
+      <c r="E41" s="37" t="s">
+        <v>167</v>
+      </c>
+      <c r="F41" s="36"/>
+      <c r="G41" s="37" t="s">
+        <v>163</v>
+      </c>
+      <c r="H41" s="36"/>
+      <c r="I41" s="36"/>
+      <c r="J41" s="67"/>
+      <c r="K41" s="70" t="s">
+        <v>165</v>
+      </c>
+      <c r="L41" s="68">
+        <v>1</v>
+      </c>
+      <c r="M41" s="36"/>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A42" s="1"/>
+      <c r="B42" s="31"/>
+      <c r="C42" s="48"/>
+      <c r="D42" s="32"/>
+      <c r="E42" s="33"/>
+      <c r="F42" s="34"/>
+      <c r="G42" s="35"/>
+      <c r="H42" s="35"/>
+      <c r="I42" s="34"/>
+      <c r="J42" s="35"/>
+      <c r="K42" s="69"/>
+      <c r="L42" s="35"/>
+      <c r="M42" s="41"/>
+    </row>
+    <row r="43" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="1"/>
+      <c r="B43" s="24"/>
+      <c r="C43" s="49"/>
+      <c r="D43" s="8"/>
+      <c r="E43" s="9"/>
+      <c r="F43" s="9"/>
+      <c r="G43" s="9"/>
+      <c r="H43" s="9"/>
+      <c r="I43" s="9"/>
+      <c r="J43" s="9"/>
+      <c r="K43" s="9"/>
+      <c r="L43" s="9"/>
+      <c r="M43" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="J1:L1"/>
-    <mergeCell ref="L3:L8"/>
+    <mergeCell ref="J1:M1"/>
+    <mergeCell ref="M3:M8"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="K39" r:id="rId1"/>
+    <hyperlink ref="K40" r:id="rId2"/>
+    <hyperlink ref="K41" r:id="rId3"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#5 eXtra peripheral link remove Client and eSpark BOM.
</commit_message>
<xml_diff>
--- a/Design Files/BLE_product-v1.0/BOM/BOM_For_BLE_product-v1.0.xlsx
+++ b/Design Files/BLE_product-v1.0/BOM/BOM_For_BLE_product-v1.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="167">
   <si>
     <t>Component list</t>
   </si>
@@ -496,9 +496,6 @@
   </si>
   <si>
     <t>Peripherals</t>
-  </si>
-  <si>
-    <t>dc2.0*0.5mm USB Charger Cable Small Pin Charging Cord</t>
   </si>
   <si>
     <t>Link</t>
@@ -933,7 +930,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1084,18 +1081,6 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1110,9 +1095,6 @@
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1123,6 +1105,15 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1466,7 +1457,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:M43"/>
+  <dimension ref="A1:M42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
@@ -1493,10 +1484,10 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="57"/>
-      <c r="K1" s="57"/>
-      <c r="L1" s="57"/>
-      <c r="M1" s="57"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="66"/>
+      <c r="L1" s="66"/>
+      <c r="M1" s="66"/>
     </row>
     <row r="2" spans="1:13" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1534,7 +1525,7 @@
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
-      <c r="M3" s="58"/>
+      <c r="M3" s="67"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1553,7 +1544,7 @@
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
       <c r="L4" s="6"/>
-      <c r="M4" s="59"/>
+      <c r="M4" s="68"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1572,7 +1563,7 @@
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
       <c r="L5" s="5"/>
-      <c r="M5" s="59"/>
+      <c r="M5" s="68"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1587,7 +1578,7 @@
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
       <c r="L6" s="5"/>
-      <c r="M6" s="59"/>
+      <c r="M6" s="68"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1602,7 +1593,7 @@
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
-      <c r="M7" s="59"/>
+      <c r="M7" s="68"/>
     </row>
     <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1617,7 +1608,7 @@
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
-      <c r="M8" s="59"/>
+      <c r="M8" s="68"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1649,7 +1640,7 @@
         <v>150</v>
       </c>
       <c r="K9" s="30" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L9" s="29" t="s">
         <v>149</v>
@@ -1688,7 +1679,7 @@
       <c r="J10" s="36" t="s">
         <v>137</v>
       </c>
-      <c r="K10" s="61"/>
+      <c r="K10" s="57"/>
       <c r="L10" s="36">
         <v>6</v>
       </c>
@@ -1724,7 +1715,7 @@
       <c r="J11" s="38" t="s">
         <v>138</v>
       </c>
-      <c r="K11" s="62"/>
+      <c r="K11" s="58"/>
       <c r="L11" s="38">
         <v>1</v>
       </c>
@@ -1760,7 +1751,7 @@
       <c r="J12" s="36" t="s">
         <v>139</v>
       </c>
-      <c r="K12" s="61"/>
+      <c r="K12" s="57"/>
       <c r="L12" s="36">
         <v>1</v>
       </c>
@@ -1796,7 +1787,7 @@
       <c r="J13" s="38" t="s">
         <v>140</v>
       </c>
-      <c r="K13" s="62"/>
+      <c r="K13" s="58"/>
       <c r="L13" s="38">
         <v>1</v>
       </c>
@@ -1832,7 +1823,7 @@
       <c r="J14" s="36" t="s">
         <v>141</v>
       </c>
-      <c r="K14" s="63"/>
+      <c r="K14" s="59"/>
       <c r="L14" s="36">
         <v>1</v>
       </c>
@@ -1868,7 +1859,7 @@
       <c r="J15" s="38" t="s">
         <v>142</v>
       </c>
-      <c r="K15" s="62"/>
+      <c r="K15" s="58"/>
       <c r="L15" s="38">
         <v>1</v>
       </c>
@@ -1904,7 +1895,7 @@
       <c r="J16" s="36" t="s">
         <v>140</v>
       </c>
-      <c r="K16" s="63"/>
+      <c r="K16" s="59"/>
       <c r="L16" s="36">
         <v>1</v>
       </c>
@@ -1944,8 +1935,8 @@
       <c r="L17" s="38">
         <v>4</v>
       </c>
-      <c r="M17" s="64" t="s">
-        <v>161</v>
+      <c r="M17" s="60" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1978,7 +1969,7 @@
       <c r="J18" s="36" t="s">
         <v>153</v>
       </c>
-      <c r="K18" s="61"/>
+      <c r="K18" s="57"/>
       <c r="L18" s="36">
         <v>1</v>
       </c>
@@ -2018,8 +2009,8 @@
       <c r="L19" s="38">
         <v>1</v>
       </c>
-      <c r="M19" s="64" t="s">
-        <v>161</v>
+      <c r="M19" s="60" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2035,13 +2026,13 @@
         <v>28</v>
       </c>
       <c r="E20" s="37" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F20" s="36" t="s">
         <v>153</v>
       </c>
       <c r="G20" s="36" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="H20" s="36" t="s">
         <v>153</v>
@@ -2052,12 +2043,12 @@
       <c r="J20" s="36" t="s">
         <v>153</v>
       </c>
-      <c r="K20" s="61"/>
+      <c r="K20" s="57"/>
       <c r="L20" s="36">
         <v>1</v>
       </c>
-      <c r="M20" s="64" t="s">
-        <v>161</v>
+      <c r="M20" s="60" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="21" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2090,7 +2081,7 @@
       <c r="J21" s="38" t="s">
         <v>143</v>
       </c>
-      <c r="K21" s="61"/>
+      <c r="K21" s="57"/>
       <c r="L21" s="38">
         <v>1</v>
       </c>
@@ -2198,7 +2189,7 @@
       <c r="J24" s="36" t="s">
         <v>144</v>
       </c>
-      <c r="K24" s="62"/>
+      <c r="K24" s="58"/>
       <c r="L24" s="36">
         <v>5</v>
       </c>
@@ -2342,7 +2333,7 @@
       <c r="J28" s="36" t="s">
         <v>148</v>
       </c>
-      <c r="K28" s="62"/>
+      <c r="K28" s="58"/>
       <c r="L28" s="36">
         <v>4</v>
       </c>
@@ -2378,7 +2369,7 @@
       <c r="J29" s="38" t="s">
         <v>153</v>
       </c>
-      <c r="K29" s="61"/>
+      <c r="K29" s="57"/>
       <c r="L29" s="38">
         <v>1</v>
       </c>
@@ -2414,7 +2405,7 @@
       <c r="J30" s="36" t="s">
         <v>153</v>
       </c>
-      <c r="K30" s="62"/>
+      <c r="K30" s="58"/>
       <c r="L30" s="36">
         <v>1</v>
       </c>
@@ -2450,7 +2441,7 @@
       <c r="J31" s="38" t="s">
         <v>153</v>
       </c>
-      <c r="K31" s="65"/>
+      <c r="K31" s="61"/>
       <c r="L31" s="38">
         <v>1</v>
       </c>
@@ -2486,7 +2477,7 @@
       <c r="J32" s="36" t="s">
         <v>153</v>
       </c>
-      <c r="K32" s="65"/>
+      <c r="K32" s="61"/>
       <c r="L32" s="36">
         <v>1</v>
       </c>
@@ -2522,7 +2513,7 @@
       <c r="J33" s="38" t="s">
         <v>153</v>
       </c>
-      <c r="K33" s="65"/>
+      <c r="K33" s="61"/>
       <c r="L33" s="38">
         <v>1</v>
       </c>
@@ -2558,7 +2549,7 @@
       <c r="J34" s="36" t="s">
         <v>153</v>
       </c>
-      <c r="K34" s="65"/>
+      <c r="K34" s="61"/>
       <c r="L34" s="36">
         <v>1</v>
       </c>
@@ -2594,7 +2585,7 @@
       <c r="J35" s="38" t="s">
         <v>153</v>
       </c>
-      <c r="K35" s="65"/>
+      <c r="K35" s="61"/>
       <c r="L35" s="38">
         <v>1</v>
       </c>
@@ -2630,7 +2621,7 @@
       <c r="J36" s="36" t="s">
         <v>153</v>
       </c>
-      <c r="K36" s="65"/>
+      <c r="K36" s="61"/>
       <c r="L36" s="36">
         <v>1</v>
       </c>
@@ -2666,7 +2657,7 @@
       <c r="J37" s="38" t="s">
         <v>153</v>
       </c>
-      <c r="K37" s="65"/>
+      <c r="K37" s="61"/>
       <c r="L37" s="38">
         <v>1</v>
       </c>
@@ -2702,15 +2693,16 @@
       <c r="J38" s="36" t="s">
         <v>153</v>
       </c>
-      <c r="K38" s="65"/>
+      <c r="K38" s="61"/>
       <c r="L38" s="36">
         <v>1</v>
       </c>
       <c r="M38" s="36"/>
     </row>
-    <row r="39" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
-      <c r="B39" s="60">
+      <c r="B39" s="50">
+        <f t="shared" ref="B39:B40" si="1">ROW(B39) - ROW($B$9)</f>
         <v>30</v>
       </c>
       <c r="C39" s="56" t="s">
@@ -2720,7 +2712,7 @@
         <v>153</v>
       </c>
       <c r="E39" s="37" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="F39" s="36" t="s">
         <v>153</v>
@@ -2732,108 +2724,74 @@
       <c r="I39" s="36" t="s">
         <v>153</v>
       </c>
-      <c r="J39" s="36" t="s">
-        <v>153</v>
-      </c>
-      <c r="K39" s="66" t="s">
-        <v>162</v>
-      </c>
-      <c r="L39" s="36">
+      <c r="J39" s="62" t="s">
+        <v>153</v>
+      </c>
+      <c r="K39" s="65" t="s">
+        <v>161</v>
+      </c>
+      <c r="L39" s="63">
         <v>1</v>
       </c>
       <c r="M39" s="36"/>
     </row>
     <row r="40" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
-      <c r="B40" s="60">
+      <c r="B40" s="50">
+        <f t="shared" si="1"/>
         <v>31</v>
       </c>
       <c r="C40" s="56" t="s">
         <v>158</v>
       </c>
-      <c r="D40" s="36" t="s">
-        <v>153</v>
-      </c>
+      <c r="D40" s="36"/>
       <c r="E40" s="37" t="s">
         <v>166</v>
       </c>
-      <c r="F40" s="36" t="s">
-        <v>153</v>
-      </c>
+      <c r="F40" s="36"/>
       <c r="G40" s="37" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="H40" s="36"/>
-      <c r="I40" s="36" t="s">
-        <v>153</v>
-      </c>
-      <c r="J40" s="67" t="s">
-        <v>153</v>
-      </c>
-      <c r="K40" s="70" t="s">
-        <v>162</v>
-      </c>
-      <c r="L40" s="68">
+      <c r="I40" s="36"/>
+      <c r="J40" s="62"/>
+      <c r="K40" s="65" t="s">
+        <v>164</v>
+      </c>
+      <c r="L40" s="63">
         <v>1</v>
       </c>
       <c r="M40" s="36"/>
     </row>
-    <row r="41" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" s="1"/>
-      <c r="B41" s="60">
-        <v>32</v>
-      </c>
-      <c r="C41" s="56" t="s">
-        <v>158</v>
-      </c>
-      <c r="D41" s="36"/>
-      <c r="E41" s="37" t="s">
-        <v>167</v>
-      </c>
-      <c r="F41" s="36"/>
-      <c r="G41" s="37" t="s">
-        <v>163</v>
-      </c>
-      <c r="H41" s="36"/>
-      <c r="I41" s="36"/>
-      <c r="J41" s="67"/>
-      <c r="K41" s="70" t="s">
-        <v>165</v>
-      </c>
-      <c r="L41" s="68">
-        <v>1</v>
-      </c>
-      <c r="M41" s="36"/>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B41" s="31"/>
+      <c r="C41" s="48"/>
+      <c r="D41" s="32"/>
+      <c r="E41" s="33"/>
+      <c r="F41" s="34"/>
+      <c r="G41" s="35"/>
+      <c r="H41" s="35"/>
+      <c r="I41" s="34"/>
+      <c r="J41" s="35"/>
+      <c r="K41" s="64"/>
+      <c r="L41" s="35"/>
+      <c r="M41" s="41"/>
+    </row>
+    <row r="42" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
-      <c r="B42" s="31"/>
-      <c r="C42" s="48"/>
-      <c r="D42" s="32"/>
-      <c r="E42" s="33"/>
-      <c r="F42" s="34"/>
-      <c r="G42" s="35"/>
-      <c r="H42" s="35"/>
-      <c r="I42" s="34"/>
-      <c r="J42" s="35"/>
-      <c r="K42" s="69"/>
-      <c r="L42" s="35"/>
-      <c r="M42" s="41"/>
-    </row>
-    <row r="43" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="1"/>
-      <c r="B43" s="24"/>
-      <c r="C43" s="49"/>
-      <c r="D43" s="8"/>
-      <c r="E43" s="9"/>
-      <c r="F43" s="9"/>
-      <c r="G43" s="9"/>
-      <c r="H43" s="9"/>
-      <c r="I43" s="9"/>
-      <c r="J43" s="9"/>
-      <c r="K43" s="9"/>
-      <c r="L43" s="9"/>
-      <c r="M43" s="42"/>
+      <c r="B42" s="24"/>
+      <c r="C42" s="49"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="9"/>
+      <c r="F42" s="9"/>
+      <c r="G42" s="9"/>
+      <c r="H42" s="9"/>
+      <c r="I42" s="9"/>
+      <c r="J42" s="9"/>
+      <c r="K42" s="9"/>
+      <c r="L42" s="9"/>
+      <c r="M42" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2843,10 +2801,9 @@
   <hyperlinks>
     <hyperlink ref="K39" r:id="rId1"/>
     <hyperlink ref="K40" r:id="rId2"/>
-    <hyperlink ref="K41" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
-  <drawing r:id="rId5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <drawing r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>